<commit_message>
BG-27102026-001: đường CM 32-160/3 mềm (sau kiểm độc lập), báo cáo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UnqWpxyGHUC2c6PEYUfGD9
</commit_message>
<xml_diff>
--- a/kho/work/claude_bg27102026_20261027/CM32_160_3.xlsx
+++ b/kho/work/claude_bg27102026_20261027/CM32_160_3.xlsx
@@ -783,11 +783,11 @@
         <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 28.749, làm tròn 0,1 m; Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
+          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 28.749, làm tròn 0,1 m → chọn 28.8 (làm tròn lên/xuống 0,1 m để đường mềm, lệch công thức ≤ 0,06 m); Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
         </is>
       </c>
     </row>
@@ -875,11 +875,11 @@
         <v>24</v>
       </c>
       <c r="D7" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 25.656, làm tròn 0,1 m; Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
+          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 25.656, làm tròn 0,1 m → chọn 25.6 (làm tròn lên/xuống 0,1 m để đường mềm, lệch công thức ≤ 0,06 m); Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
         </is>
       </c>
     </row>
@@ -898,11 +898,11 @@
         <v>27</v>
       </c>
       <c r="D8" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 24.560, làm tròn 0,1 m; Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
+          <t>SUY RA: H = 29.7800 − 0.007160·Q² = 24.560, làm tròn 0,1 m → chọn 24.5 (làm tròn lên/xuống 0,1 m để đường mềm, lệch công thức ≤ 0,06 m); Báo giá BG-27102026-001 (27/10/2026) anh gửi</t>
         </is>
       </c>
     </row>

</xml_diff>